<commit_message>
Sessions by number, not clock time; venue and contact e-mail filled in
Decks and participant handouts now say 'Session 1' to 'Session 8' instead of
09:40, 10:00 and so on, so the day can run late without contradicting anything
in a participant's hand. The facilitator run sheet keeps a clock column.

Brochure and agenda rebuilt with the venue room (Samvad, Board Room) and the
confirmed contact address hta@aiimsbhopal.edu.in. Both pages still fit 297 mm.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LFbbEuXWcteyzCrQZnfwXc
</commit_message>
<xml_diff>
--- a/handouts/poll-bank.xlsx
+++ b/handouts/poll-bank.xlsx
@@ -445,12 +445,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Session time</t>
+          <t>Session</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Session</t>
+          <t>Topic</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>Session 1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -541,7 +541,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Baseline only. Re-ask at 16:20 in a different form (the confidence question).</t>
+          <t>Baseline only. Re-ask at the close in a different form (the confidence question).</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>Session 1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>Session 3</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>Session 3</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Chugh et al. 2026. ₹54,881 is the ICER for VIA screening from Block 1, a distractor on purpose.</t>
+          <t>Chugh et al. 2026. ₹54,881 is the ICER for VIA screening from Session 2, a distractor on purpose.</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>Session 3</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>Session 4</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>Session 4</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>Session 4</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>Session 5</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>Session 5</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>12:35</t>
+          <t>Session 5</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>Session 6</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>Session 6</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>3,400 ÷ 0.13. ₹204 is the average ratio from Block 3B: total cost over total QALYs, meaningless for a decision.</t>
+          <t>3,400 ÷ 0.13. ₹204 is the average ratio from Session 6: total cost over total QALYs, meaningless for a decision.</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>Session 6</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>Session 7</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>Session 7</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>Session 8</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>Session 8</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>Session 8</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Compare with the 09:40 baseline. Opinion; no right answer.</t>
+          <t>Compare with the Session 1 baseline. Opinion; no right answer.</t>
         </is>
       </c>
     </row>

</xml_diff>